<commit_message>
Add Windows GUI and other tweaks
</commit_message>
<xml_diff>
--- a/artifacts/Sep21_Oct18_Schedule.xlsx
+++ b/artifacts/Sep21_Oct18_Schedule.xlsx
@@ -713,7 +713,11 @@
       <c r="G2" s="5" t="n"/>
       <c r="H2" s="5" t="n"/>
       <c r="I2" s="5" t="n"/>
-      <c r="J2" s="5" t="n"/>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>8-8</t>
+        </is>
+      </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
           <t>2-12</t>
@@ -721,52 +725,48 @@
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>O/N</t>
-        </is>
-      </c>
-      <c r="M2" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="n"/>
       <c r="N2" s="5" t="n"/>
       <c r="O2" s="5" t="n"/>
       <c r="P2" s="5" t="n"/>
-      <c r="Q2" s="5" t="n"/>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
       <c r="R2" s="5" t="inlineStr">
         <is>
-          <t>8-6</t>
+          <t>O/N</t>
         </is>
       </c>
       <c r="S2" s="5" t="inlineStr">
         <is>
-          <t>8-8</t>
-        </is>
-      </c>
-      <c r="T2" s="5" t="inlineStr">
-        <is>
-          <t>2-12</t>
-        </is>
-      </c>
+          <t>O/N</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="n"/>
       <c r="U2" s="5" t="n"/>
       <c r="V2" s="5" t="n"/>
-      <c r="W2" s="5" t="inlineStr">
-        <is>
-          <t>2-12</t>
-        </is>
-      </c>
-      <c r="X2" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
+      <c r="W2" s="5" t="n"/>
+      <c r="X2" s="5" t="n"/>
       <c r="Y2" s="5" t="inlineStr">
         <is>
-          <t>O/N</t>
-        </is>
-      </c>
-      <c r="Z2" s="5" t="n"/>
-      <c r="AA2" s="5" t="n"/>
+          <t>8-8</t>
+        </is>
+      </c>
+      <c r="Z2" s="5" t="inlineStr">
+        <is>
+          <t>O/N</t>
+        </is>
+      </c>
+      <c r="AA2" s="5" t="inlineStr">
+        <is>
+          <t>O/N</t>
+        </is>
+      </c>
       <c r="AB2" s="5" t="n"/>
       <c r="AC2" s="5" t="n"/>
     </row>
@@ -776,14 +776,26 @@
           <t>Meaghan</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
       <c r="D3" s="5" t="n"/>
       <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>8-8</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>2-12</t>
+          <t>O/N</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
@@ -791,67 +803,55 @@
           <t>O/N</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
+      <c r="I3" s="5" t="n"/>
       <c r="J3" s="5" t="n"/>
       <c r="K3" s="5" t="n"/>
       <c r="L3" s="5" t="n"/>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>8-6</t>
+          <t>2-12</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
-          <t>8-8</t>
-        </is>
-      </c>
-      <c r="O3" s="5" t="n"/>
-      <c r="P3" s="5" t="inlineStr">
-        <is>
-          <t>8-8</t>
-        </is>
-      </c>
+          <t>O/N</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>O/N</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="n"/>
       <c r="Q3" s="5" t="n"/>
       <c r="R3" s="5" t="n"/>
       <c r="S3" s="5" t="inlineStr">
         <is>
-          <t>2-12</t>
+          <t>8-8</t>
         </is>
       </c>
       <c r="T3" s="5" t="inlineStr">
         <is>
-          <t>O/N</t>
-        </is>
-      </c>
-      <c r="U3" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="n"/>
       <c r="V3" s="5" t="n"/>
       <c r="W3" s="5" t="n"/>
-      <c r="X3" s="5" t="n"/>
-      <c r="Y3" s="5" t="n"/>
+      <c r="X3" s="5" t="inlineStr">
+        <is>
+          <t>O/N</t>
+        </is>
+      </c>
+      <c r="Y3" s="5" t="inlineStr">
+        <is>
+          <t>O/N</t>
+        </is>
+      </c>
       <c r="Z3" s="5" t="n"/>
-      <c r="AA3" s="5" t="inlineStr">
-        <is>
-          <t>2-12</t>
-        </is>
-      </c>
-      <c r="AB3" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
-      <c r="AC3" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
+      <c r="AA3" s="5" t="n"/>
+      <c r="AB3" s="5" t="n"/>
+      <c r="AC3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -859,79 +859,79 @@
           <t>Katherine</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>2-12</t>
-        </is>
-      </c>
+      <c r="B4" s="5" t="n"/>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>2-12</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="n"/>
+          <t>O/N</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>O/N</t>
+        </is>
+      </c>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>2-12</t>
-        </is>
-      </c>
+      <c r="H4" s="5" t="n"/>
       <c r="I4" s="5" t="inlineStr">
         <is>
           <t>2-12</t>
         </is>
       </c>
-      <c r="J4" s="5" t="n"/>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
       <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="inlineStr">
-        <is>
-          <t>2-12</t>
-        </is>
-      </c>
+      <c r="L4" s="5" t="n"/>
       <c r="M4" s="5" t="n"/>
-      <c r="N4" s="5" t="n"/>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>8-6</t>
+          <t>2-12</t>
         </is>
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>O/N</t>
-        </is>
-      </c>
-      <c r="Q4" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="Q4" s="5" t="n"/>
       <c r="R4" s="5" t="n"/>
       <c r="S4" s="5" t="n"/>
-      <c r="T4" s="5" t="n"/>
+      <c r="T4" s="5" t="inlineStr">
+        <is>
+          <t>8-8</t>
+        </is>
+      </c>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>8-6</t>
-        </is>
-      </c>
-      <c r="V4" s="5" t="inlineStr">
-        <is>
-          <t>8-6</t>
-        </is>
-      </c>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="V4" s="5" t="n"/>
       <c r="W4" s="5" t="n"/>
-      <c r="X4" s="5" t="n"/>
-      <c r="Y4" s="5" t="n"/>
-      <c r="Z4" s="5" t="inlineStr">
-        <is>
-          <t>8-8</t>
-        </is>
-      </c>
+      <c r="X4" s="5" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="Y4" s="5" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="Z4" s="5" t="n"/>
       <c r="AA4" s="5" t="n"/>
       <c r="AB4" s="5" t="inlineStr">
         <is>
-          <t>8-6</t>
+          <t>2-12</t>
         </is>
       </c>
       <c r="AC4" s="5" t="inlineStr">
@@ -946,56 +946,56 @@
           <t>Kristyne</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>8-6</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
           <t>O/N</t>
         </is>
       </c>
-      <c r="F5" s="5" t="n"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>O/N</t>
+        </is>
+      </c>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
       <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>8-8</t>
-        </is>
-      </c>
+      <c r="J5" s="5" t="n"/>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>8-8</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="n"/>
-      <c r="M5" s="5" t="n"/>
-      <c r="N5" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
-      <c r="O5" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
+          <t>O/N</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>O/N</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>O/N</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="n"/>
+      <c r="O5" s="5" t="n"/>
       <c r="P5" s="5" t="n"/>
       <c r="Q5" s="5" t="n"/>
       <c r="R5" s="5" t="n"/>
       <c r="S5" s="5" t="n"/>
-      <c r="T5" s="5" t="n"/>
+      <c r="T5" s="5" t="inlineStr">
+        <is>
+          <t>8-6</t>
+        </is>
+      </c>
       <c r="U5" s="5" t="inlineStr">
         <is>
-          <t>2-12</t>
+          <t>8-6</t>
         </is>
       </c>
       <c r="V5" s="5" t="inlineStr">
@@ -1005,21 +1005,21 @@
       </c>
       <c r="W5" s="5" t="n"/>
       <c r="X5" s="5" t="n"/>
-      <c r="Y5" s="5" t="inlineStr">
-        <is>
-          <t>8-8</t>
-        </is>
-      </c>
+      <c r="Y5" s="5" t="n"/>
       <c r="Z5" s="5" t="inlineStr">
         <is>
-          <t>2-12</t>
+          <t>8-8</t>
         </is>
       </c>
       <c r="AA5" s="5" t="n"/>
-      <c r="AB5" s="5" t="n"/>
+      <c r="AB5" s="5" t="inlineStr">
+        <is>
+          <t>8-8</t>
+        </is>
+      </c>
       <c r="AC5" s="5" t="inlineStr">
         <is>
-          <t>8-6</t>
+          <t>8-8</t>
         </is>
       </c>
     </row>
@@ -1033,16 +1033,16 @@
       <c r="C6" s="5" t="n"/>
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>8-8</t>
-        </is>
-      </c>
+      <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>8-6</t>
+          <t>O/N</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -1050,59 +1050,59 @@
           <t>O/N</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
+      <c r="K6" s="5" t="n"/>
       <c r="L6" s="5" t="n"/>
       <c r="M6" s="5" t="n"/>
-      <c r="N6" s="5" t="n"/>
-      <c r="O6" s="5" t="n"/>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>8-8</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>8-8</t>
+        </is>
+      </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>2-12</t>
-        </is>
-      </c>
-      <c r="Q6" s="5" t="inlineStr">
-        <is>
-          <t>2-12</t>
-        </is>
-      </c>
-      <c r="R6" s="5" t="inlineStr">
-        <is>
-          <t>2-12</t>
-        </is>
-      </c>
-      <c r="S6" s="5" t="n"/>
-      <c r="T6" s="5" t="n"/>
+          <t>8-8</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="n"/>
+      <c r="R6" s="5" t="n"/>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>8-6</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr">
+        <is>
+          <t>O/N</t>
+        </is>
+      </c>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>8-8</t>
-        </is>
-      </c>
-      <c r="V6" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
-      <c r="W6" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
+          <t>O/N</t>
+        </is>
+      </c>
+      <c r="V6" s="5" t="n"/>
+      <c r="W6" s="5" t="n"/>
       <c r="X6" s="5" t="n"/>
       <c r="Y6" s="5" t="n"/>
       <c r="Z6" s="5" t="n"/>
-      <c r="AA6" s="5" t="n"/>
+      <c r="AA6" s="5" t="inlineStr">
+        <is>
+          <t>8-6</t>
+        </is>
+      </c>
       <c r="AB6" s="5" t="inlineStr">
         <is>
-          <t>8-8</t>
+          <t>8-6</t>
         </is>
       </c>
       <c r="AC6" s="5" t="inlineStr">
         <is>
-          <t>8-8</t>
+          <t>8-6</t>
         </is>
       </c>
     </row>
@@ -1112,82 +1112,82 @@
           <t>Sydney</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>8-8</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>8-8</t>
-        </is>
-      </c>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
       <c r="D7" s="5" t="n"/>
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>O/N</t>
+          <t>8-6</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>O/N</t>
+          <t>2-12</t>
         </is>
       </c>
       <c r="H7" s="5" t="n"/>
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="n"/>
       <c r="K7" s="5" t="n"/>
-      <c r="L7" s="5" t="n"/>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>8-6</t>
+        </is>
+      </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>2-12</t>
-        </is>
-      </c>
-      <c r="N7" s="5" t="inlineStr">
-        <is>
-          <t>2-12</t>
-        </is>
-      </c>
-      <c r="O7" s="5" t="inlineStr">
-        <is>
-          <t>2-12</t>
-        </is>
-      </c>
-      <c r="P7" s="5" t="n"/>
-      <c r="Q7" s="5" t="n"/>
-      <c r="R7" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
-      <c r="S7" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
+          <t>8-6</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="n"/>
+      <c r="O7" s="5" t="n"/>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>O/N</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>O/N</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="n"/>
+      <c r="S7" s="5" t="n"/>
       <c r="T7" s="5" t="n"/>
-      <c r="U7" s="5" t="n"/>
-      <c r="V7" s="5" t="n"/>
-      <c r="W7" s="5" t="n"/>
+      <c r="U7" s="5" t="inlineStr">
+        <is>
+          <t>8-8</t>
+        </is>
+      </c>
+      <c r="V7" s="5" t="inlineStr">
+        <is>
+          <t>O/N</t>
+        </is>
+      </c>
+      <c r="W7" s="5" t="inlineStr">
+        <is>
+          <t>O/N</t>
+        </is>
+      </c>
       <c r="X7" s="5" t="n"/>
-      <c r="Y7" s="5" t="inlineStr">
-        <is>
-          <t>2-12</t>
-        </is>
-      </c>
-      <c r="Z7" s="5" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
+      <c r="Y7" s="5" t="n"/>
+      <c r="Z7" s="5" t="n"/>
       <c r="AA7" s="5" t="inlineStr">
         <is>
-          <t>O/N</t>
-        </is>
-      </c>
-      <c r="AB7" s="5" t="n"/>
-      <c r="AC7" s="5" t="n"/>
+          <t>8-8</t>
+        </is>
+      </c>
+      <c r="AB7" s="5" t="inlineStr">
+        <is>
+          <t>O/N</t>
+        </is>
+      </c>
+      <c r="AC7" s="5" t="inlineStr">
+        <is>
+          <t>O/N</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1271,12 +1271,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>8-6</t>
+          <t>8-8</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>8-6</t>
+          <t>8-8</t>
         </is>
       </c>
       <c r="D10" s="5" t="n"/>
@@ -1293,12 +1293,12 @@
         </is>
       </c>
       <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>2-12</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="n"/>
+      <c r="J10" s="5" t="n"/>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>8-8</t>
+        </is>
+      </c>
       <c r="L10" s="5" t="n"/>
       <c r="M10" s="5" t="n"/>
       <c r="N10" s="5" t="inlineStr">
@@ -1308,46 +1308,46 @@
       </c>
       <c r="O10" s="5" t="inlineStr">
         <is>
-          <t>8-8</t>
+          <t>8-6</t>
         </is>
       </c>
       <c r="P10" s="5" t="n"/>
       <c r="Q10" s="5" t="n"/>
-      <c r="R10" s="5" t="n"/>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>8-6</t>
-        </is>
-      </c>
-      <c r="T10" s="5" t="inlineStr">
-        <is>
-          <t>8-8</t>
-        </is>
-      </c>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="T10" s="5" t="n"/>
       <c r="U10" s="5" t="n"/>
-      <c r="V10" s="5" t="n"/>
+      <c r="V10" s="5" t="inlineStr">
+        <is>
+          <t>8-6</t>
+        </is>
+      </c>
       <c r="W10" s="5" t="inlineStr">
         <is>
-          <t>8-6</t>
-        </is>
-      </c>
-      <c r="X10" s="5" t="inlineStr">
-        <is>
-          <t>2-12</t>
-        </is>
-      </c>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="X10" s="5" t="n"/>
       <c r="Y10" s="5" t="n"/>
-      <c r="Z10" s="5" t="n"/>
+      <c r="Z10" s="5" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
       <c r="AA10" s="5" t="inlineStr">
         <is>
-          <t>8-8</t>
-        </is>
-      </c>
-      <c r="AB10" s="5" t="inlineStr">
-        <is>
-          <t>2-12</t>
-        </is>
-      </c>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="AB10" s="5" t="n"/>
       <c r="AC10" s="5" t="n"/>
     </row>
     <row r="11">
@@ -1357,7 +1357,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>8-6</t>
+        </is>
+      </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
           <t>8-6</t>
@@ -1368,14 +1372,14 @@
           <t>8-6</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>8-6</t>
-        </is>
-      </c>
+      <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="n"/>
       <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>8-6</t>
+        </is>
+      </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
           <t>8-6</t>
@@ -1386,11 +1390,7 @@
           <t>8-6</t>
         </is>
       </c>
-      <c r="L11" s="5" t="inlineStr">
-        <is>
-          <t>8-6</t>
-        </is>
-      </c>
+      <c r="L11" s="5" t="n"/>
       <c r="M11" s="5" t="n"/>
       <c r="N11" s="5" t="n"/>
       <c r="O11" s="5" t="n"/>
@@ -1404,16 +1404,20 @@
           <t>8-6</t>
         </is>
       </c>
-      <c r="R11" s="5" t="n"/>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>8-6</t>
+        </is>
+      </c>
       <c r="S11" s="5" t="n"/>
-      <c r="T11" s="5" t="inlineStr">
-        <is>
-          <t>8-6</t>
-        </is>
-      </c>
+      <c r="T11" s="5" t="n"/>
       <c r="U11" s="5" t="n"/>
       <c r="V11" s="5" t="n"/>
-      <c r="W11" s="5" t="n"/>
+      <c r="W11" s="5" t="inlineStr">
+        <is>
+          <t>8-6</t>
+        </is>
+      </c>
       <c r="X11" s="5" t="inlineStr">
         <is>
           <t>8-6</t>
@@ -1429,11 +1433,7 @@
           <t>8-6</t>
         </is>
       </c>
-      <c r="AA11" s="5" t="inlineStr">
-        <is>
-          <t>8-6</t>
-        </is>
-      </c>
+      <c r="AA11" s="5" t="n"/>
       <c r="AB11" s="5" t="n"/>
       <c r="AC11" s="5" t="n"/>
     </row>
@@ -1670,10 +1670,10 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2" s="8" t="n">
         <v>4</v>
@@ -1688,13 +1688,13 @@
         <v>16</v>
       </c>
       <c r="I2" s="8" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="J2" s="8" t="n">
         <v>120</v>
       </c>
       <c r="K2" s="8" t="n">
-        <v>33.5</v>
+        <v>34</v>
       </c>
       <c r="L2" s="8" t="n">
         <v>0</v>
@@ -1718,13 +1718,13 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F3" s="8" t="n">
         <v>6</v>
@@ -1745,7 +1745,7 @@
         <v>34</v>
       </c>
       <c r="L3" s="8" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M3" s="8" t="n">
         <v>4</v>
@@ -1766,13 +1766,13 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>2</v>
@@ -1793,7 +1793,7 @@
         <v>34</v>
       </c>
       <c r="L4" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M4" s="8" t="n">
         <v>2</v>
@@ -1814,13 +1814,13 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F5" s="8" t="n">
         <v>5</v>
@@ -1841,7 +1841,7 @@
         <v>34</v>
       </c>
       <c r="L5" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M5" s="8" t="n">
         <v>5</v>
@@ -1862,13 +1862,13 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="8" t="n">
         <v>1</v>
-      </c>
-      <c r="D6" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E6" s="8" t="n">
-        <v>3</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>4</v>
@@ -1880,16 +1880,16 @@
         <v>16</v>
       </c>
       <c r="I6" s="8" t="n">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J6" s="8" t="n">
         <v>120</v>
       </c>
       <c r="K6" s="8" t="n">
-        <v>34</v>
+        <v>33.5</v>
       </c>
       <c r="L6" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M6" s="8" t="n">
         <v>6</v>
@@ -1910,13 +1910,13 @@
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F7" s="8" t="n">
         <v>6</v>
@@ -1937,7 +1937,7 @@
         <v>34</v>
       </c>
       <c r="L7" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M7" s="8" t="n">
         <v>4</v>
@@ -2054,13 +2054,13 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>3</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>0</v>
@@ -2350,7 +2350,7 @@
         <v>5330667</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>0.982</v>
+        <v>1.051</v>
       </c>
     </row>
     <row r="9">
@@ -2368,7 +2368,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>0.364</v>
+        <v>0.407</v>
       </c>
     </row>
     <row r="10">
@@ -2383,10 +2383,10 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>41952</v>
+        <v>31872</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>30.027</v>
+        <v>60.023</v>
       </c>
     </row>
     <row r="11"/>

</xml_diff>